<commit_message>
justPipe on MVP pattern v3; 11/08/2026 further developments (Added pt snapping on not visited; removed not visited)
</commit_message>
<xml_diff>
--- a/project/_src/_internal/config/DatStructures.xlsx
+++ b/project/_src/_internal/config/DatStructures.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AK\PyProj\jP\JustPipe\project\_src\_internal\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{13F788C9-969D-49EC-8323-114A741EE044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A72F21CA-7B74-4E71-9BBB-A275FFC5D488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F4D73261-E1E9-4FDB-8B2D-DEB2BE8DE16F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="126">
   <si>
     <t>"_x000D_
 EIVA EXPORT STRING:_x000D_
@@ -279,9 +279,6 @@
     <t xml:space="preserve">        29: POI flag</t>
   </si>
   <si>
-    <t xml:space="preserve">        30: visited flag diff (for plotting visited parts)</t>
-  </si>
-  <si>
     <t xml:space="preserve">    'pipetracker':</t>
   </si>
   <si>
@@ -415,16 +412,32 @@
   </si>
   <si>
     <t xml:space="preserve">        RMB - select chunk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        14: shifted easting by statistic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        15: shifted northing by statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        30: digitized by pipe(1)/pipetracker(0)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -450,11 +463,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -789,7 +803,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE9FDC0A-FC46-4597-8379-FC44A6DC036F}">
-  <dimension ref="A1:F145"/>
+  <dimension ref="A1:F147"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1203,257 +1217,267 @@
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>78</v>
+      <c r="A92" s="2" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>93</v>
+        <v>92</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A109" s="2" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>3</v>
+      <c r="A110" s="2" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>99</v>
+        <v>25</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>102</v>
+        <v>99</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>